<commit_message>
New gas meters isntalled
</commit_message>
<xml_diff>
--- a/data/Summer_Ridge_Master_Sheet.xlsx
+++ b/data/Summer_Ridge_Master_Sheet.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Summer Ridge/Estate Management/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="140" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67098C37-D966-4BF4-91BF-B7E28FD8FF2C}"/>
+  <xr:revisionPtr revIDLastSave="188" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9FB7259-DE41-44B7-8893-534D3CAF51D4}"/>
   <bookViews>
-    <workbookView xWindow="71880" yWindow="-1530" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
+    <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
     <sheet name="Gas" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Gas!$A$1:$C$152</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -635,7 +638,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -3746,7 +3760,7 @@
         <v>25003273</v>
       </c>
       <c r="C2" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
@@ -3757,7 +3771,7 @@
         <v>25003187</v>
       </c>
       <c r="C3" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
@@ -3790,7 +3804,7 @@
         <v>25003302</v>
       </c>
       <c r="C6" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.45">
@@ -3812,7 +3826,7 @@
         <v>25003167</v>
       </c>
       <c r="C8" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
@@ -3845,7 +3859,7 @@
         <v>25003183</v>
       </c>
       <c r="C11" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.45">
@@ -3878,7 +3892,7 @@
         <v>25003188</v>
       </c>
       <c r="C14" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.45">
@@ -3889,7 +3903,7 @@
         <v>25003184</v>
       </c>
       <c r="C15" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.45">
@@ -3900,7 +3914,7 @@
         <v>25003218</v>
       </c>
       <c r="C16" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.45">
@@ -3911,7 +3925,7 @@
         <v>25003212</v>
       </c>
       <c r="C17" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.45">
@@ -3922,7 +3936,7 @@
         <v>25003164</v>
       </c>
       <c r="C18" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.45">
@@ -3933,7 +3947,7 @@
         <v>25003197</v>
       </c>
       <c r="C19" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.45">
@@ -3955,7 +3969,7 @@
         <v>25000769</v>
       </c>
       <c r="C21" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.45">
@@ -4010,7 +4024,7 @@
         <v>25003228</v>
       </c>
       <c r="C26" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.45">
@@ -4054,7 +4068,7 @@
         <v>25003225</v>
       </c>
       <c r="C30" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.45">
@@ -4076,7 +4090,7 @@
         <v>25003208</v>
       </c>
       <c r="C32" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.45">
@@ -4164,7 +4178,7 @@
         <v>25003207</v>
       </c>
       <c r="C40" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.45">
@@ -4186,7 +4200,7 @@
         <v>25003244</v>
       </c>
       <c r="C42" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.45">
@@ -4208,7 +4222,7 @@
         <v>25003253</v>
       </c>
       <c r="C44" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.45">
@@ -4230,7 +4244,7 @@
         <v>25003201</v>
       </c>
       <c r="C46" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.45">
@@ -5400,6 +5414,9 @@
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B2:B152">
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
new gas meters installed
</commit_message>
<xml_diff>
--- a/data/Summer_Ridge_Master_Sheet.xlsx
+++ b/data/Summer_Ridge_Master_Sheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Summer Ridge/Estate Management/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Summer Ridge/Estate Management/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="188" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9FB7259-DE41-44B7-8893-534D3CAF51D4}"/>
+  <xr:revisionPtr revIDLastSave="194" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{46CF412B-1059-416F-A712-6B96005F6DF0}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
   </bookViews>
@@ -20,6 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Gas!$A$1:$C$152</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -4112,7 +4113,7 @@
         <v>25003168</v>
       </c>
       <c r="C34" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.45">
@@ -4123,7 +4124,7 @@
         <v>25003191</v>
       </c>
       <c r="C35" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.45">
@@ -4134,7 +4135,7 @@
         <v>25003189</v>
       </c>
       <c r="C36" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.45">
@@ -4156,7 +4157,7 @@
         <v>25003170</v>
       </c>
       <c r="C38" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.45">
@@ -4189,7 +4190,7 @@
         <v>25003229</v>
       </c>
       <c r="C41" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.45">
@@ -4310,7 +4311,7 @@
         <v>25003163</v>
       </c>
       <c r="C52" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
new gas devices installed floor 3
</commit_message>
<xml_diff>
--- a/data/Summer_Ridge_Master_Sheet.xlsx
+++ b/data/Summer_Ridge_Master_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Summer Ridge/Estate Management/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="195" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B7ABC99-927F-4485-B42B-A9BE482410FC}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB69F5CA-BD29-479A-B3A7-F2F42047B2AA}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="-7455" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
   </bookViews>
   <sheets>
     <sheet name="Elec" sheetId="1" r:id="rId1"/>
@@ -4168,7 +4168,7 @@
         <v>25003213</v>
       </c>
       <c r="C39" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.45">
@@ -4344,7 +4344,7 @@
         <v>25003298</v>
       </c>
       <c r="C55" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.45">
@@ -4366,7 +4366,7 @@
         <v>25003242</v>
       </c>
       <c r="C57" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.45">
@@ -4377,7 +4377,7 @@
         <v>25003264</v>
       </c>
       <c r="C58" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.45">
@@ -4421,7 +4421,7 @@
         <v>25003294</v>
       </c>
       <c r="C62" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.45">
@@ -4432,7 +4432,7 @@
         <v>25003196</v>
       </c>
       <c r="C63" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.45">
@@ -4465,7 +4465,7 @@
         <v>25003230</v>
       </c>
       <c r="C66" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.45">
@@ -4487,7 +4487,7 @@
         <v>25003198</v>
       </c>
       <c r="C68" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.45">
@@ -4498,7 +4498,7 @@
         <v>25003174</v>
       </c>
       <c r="C69" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.45">
@@ -4520,7 +4520,7 @@
         <v>25003268</v>
       </c>
       <c r="C71" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.45">
@@ -4531,7 +4531,7 @@
         <v>25003300</v>
       </c>
       <c r="C72" s="6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Floor 6 meters installed
</commit_message>
<xml_diff>
--- a/data/Summer_Ridge_Master_Sheet.xlsx
+++ b/data/Summer_Ridge_Master_Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://voltano-my.sharepoint.com/personal/ruan_vh_voltano_com/Documents/Desktop/Voltano/Clients/Summer Ridge/Estate Management/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="397" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{576350ED-3991-4673-8098-F4B5F1ACF6CB}"/>
+  <xr:revisionPtr revIDLastSave="472" documentId="8_{61B75D5B-E2B9-4A15-B62A-CAAC6678E594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{837F13BA-D686-4679-86CA-F8DC7EECE728}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{97778EF9-769A-4231-8D2B-397889BE3400}"/>
   </bookViews>
@@ -4044,9 +4044,11 @@
         <v>25003301</v>
       </c>
       <c r="C22" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D22" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
@@ -4400,9 +4402,11 @@
         <v>25003205</v>
       </c>
       <c r="C48" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D48" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D48" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
@@ -4412,9 +4416,11 @@
         <v>25003293</v>
       </c>
       <c r="C49" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D49" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D49" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
@@ -4558,7 +4564,7 @@
         <v>25003257</v>
       </c>
       <c r="C60" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D60" s="5">
         <v>46224</v>
@@ -4756,9 +4762,11 @@
         <v>25003309</v>
       </c>
       <c r="C75" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D75" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D75" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
@@ -4810,9 +4818,11 @@
         <v>25003285</v>
       </c>
       <c r="C79" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D79" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D79" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
@@ -4822,9 +4832,11 @@
         <v>25003192</v>
       </c>
       <c r="C80" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D80" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D80" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
@@ -4848,9 +4860,11 @@
         <v>25003240</v>
       </c>
       <c r="C82" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D82" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D82" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
@@ -4860,9 +4874,11 @@
         <v>25003194</v>
       </c>
       <c r="C83" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D83" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D83" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A84" s="2" t="s">
@@ -4872,9 +4888,11 @@
         <v>25003224</v>
       </c>
       <c r="C84" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D84" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D84" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A85" s="2" t="s">
@@ -4910,9 +4928,11 @@
         <v>25003258</v>
       </c>
       <c r="C87" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D87" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D87" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A88" s="2" t="s">
@@ -5014,9 +5034,11 @@
         <v>25003232</v>
       </c>
       <c r="C95" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D95" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D95" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A96" s="2" t="s">
@@ -5040,9 +5062,11 @@
         <v>25003193</v>
       </c>
       <c r="C97" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D97" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D97" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A98" s="2" t="s">
@@ -5114,9 +5138,11 @@
         <v>25003237</v>
       </c>
       <c r="C103" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D103" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D103" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A104" s="2" t="s">
@@ -5126,9 +5152,11 @@
         <v>25003260</v>
       </c>
       <c r="C104" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D104" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D104" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A105" s="2" t="s">
@@ -5138,9 +5166,11 @@
         <v>25003307</v>
       </c>
       <c r="C105" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D105" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D105" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A106" s="2" t="s">
@@ -5164,9 +5194,11 @@
         <v>25003279</v>
       </c>
       <c r="C107" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D107" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D107" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A108" s="2" t="s">
@@ -5188,9 +5220,11 @@
         <v>25003275</v>
       </c>
       <c r="C109" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D109" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D109" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A110" s="2" t="s">
@@ -5200,9 +5234,11 @@
         <v>25003255</v>
       </c>
       <c r="C110" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D110" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D110" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A111" s="2" t="s">
@@ -5226,9 +5262,11 @@
         <v>25003233</v>
       </c>
       <c r="C112" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D112" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D112" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A113" s="2" t="s">
@@ -5238,9 +5276,11 @@
         <v>25003262</v>
       </c>
       <c r="C113" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D113" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D113" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A114" s="2" t="s">
@@ -5250,9 +5290,11 @@
         <v>25003271</v>
       </c>
       <c r="C114" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D114" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D114" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A115" s="2" t="s">
@@ -5274,9 +5316,11 @@
         <v>25003231</v>
       </c>
       <c r="C116" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D116" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D116" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A117" s="2" t="s">
@@ -5286,9 +5330,11 @@
         <v>25003312</v>
       </c>
       <c r="C117" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D117" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D117" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A118" s="2" t="s">
@@ -5312,9 +5358,11 @@
         <v>25003296</v>
       </c>
       <c r="C119" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D119" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D119" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A120" s="2" t="s">
@@ -5324,9 +5372,11 @@
         <v>25003295</v>
       </c>
       <c r="C120" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D120" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D120" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A121" s="2" t="s">
@@ -5336,9 +5386,11 @@
         <v>25003249</v>
       </c>
       <c r="C121" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D121" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D121" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A122" s="2" t="s">
@@ -5348,9 +5400,11 @@
         <v>25003282</v>
       </c>
       <c r="C122" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D122" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D122" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A123" s="2" t="s">
@@ -5360,9 +5414,11 @@
         <v>25003310</v>
       </c>
       <c r="C123" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D123" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D123" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A124" s="2" t="s">
@@ -5410,9 +5466,11 @@
         <v>25003278</v>
       </c>
       <c r="C127" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D127" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D127" s="5">
+        <v>46225</v>
+      </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A128" s="2" t="s">
@@ -5446,9 +5504,11 @@
         <v>25003277</v>
       </c>
       <c r="C130" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D130" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D130" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A131" s="2" t="s">
@@ -5458,9 +5518,11 @@
         <v>25003281</v>
       </c>
       <c r="C131" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D131" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D131" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A132" s="2" t="s">
@@ -5510,9 +5572,11 @@
         <v>25003204</v>
       </c>
       <c r="C135" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D135" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D135" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A136" s="2" t="s">
@@ -5522,9 +5586,11 @@
         <v>25003263</v>
       </c>
       <c r="C136" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D136" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D136" s="5">
+        <v>46227</v>
+      </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A137" s="2" t="s">
@@ -5708,9 +5774,11 @@
         <v>25003288</v>
       </c>
       <c r="C151" s="4" t="b">
-        <v>0</v>
-      </c>
-      <c r="D151" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="D151" s="5">
+        <v>46226</v>
+      </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A152" s="2" t="s">

</xml_diff>